<commit_message>
added extra entry in test_data Excel file
</commit_message>
<xml_diff>
--- a/test_data/Users.xlsx
+++ b/test_data/Users.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sidharath\source\repos\CI Automation\test_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33B5CB7A-CB32-4B8D-B0F8-086CF3692C72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B195330-302D-4EA4-B894-9C5C5E3BCED9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="2316" windowWidth="21636" windowHeight="9876" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>username</t>
   </si>
@@ -43,13 +43,16 @@
   </si>
   <si>
     <t>devv@1234567</t>
+  </si>
+  <si>
+    <t>rachel_spa2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -61,6 +64,12 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -371,7 +380,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.5546875" customWidth="1"/>
@@ -402,7 +411,13 @@
         <v>5</v>
       </c>
     </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" xr:uid="{445E876F-5A40-496F-8AC4-CCFE3576E8BC}"/>
     <hyperlink ref="B3" r:id="rId2" xr:uid="{07342383-6D7A-41E6-8DD2-A6CB3E66C427}"/>

</xml_diff>